<commit_message>
Update prepared sentences with unique sentences
</commit_message>
<xml_diff>
--- a/Sentences/prepared_sentences.xlsx
+++ b/Sentences/prepared_sentences.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="302">
   <si>
     <t xml:space="preserve">Indeks zadnia </t>
   </si>
@@ -476,6 +476,456 @@
   </si>
   <si>
     <t xml:space="preserve">Zmęczony pies nie chce dzisiaj pić i jeść.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nie, on dzisiaj nie ma pieniędzy na nowy telefon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Przepraszam, że ja nie chciałem wczoraj pomóc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego my nie mamy dzisiaj gorącej kawy?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co ty chcesz robić jutro wieczorem w domu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My jesteśmy dzisiaj weseli, bo mamy dużo czasu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dziękuję za wczoraj, to był bardzo dobry dzień.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zawsze mam dobry pomysł na nową książkę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nie mam teraz czasu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jestem zmęczony więc idę spać.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nie mam jutro urodzin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gdzie jest mój klucz?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brat ma nowy samochód.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Twoja siostra jest bardzo wesoła.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Babcia i dziadek są w domu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moja siostra ma małego psa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wczoraj był dobry dzień.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dzisiaj jest poniedziałek.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Który dzisiaj jest rok?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co robisz rano?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gdzie jest twój telefon?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kto ma mój klucz?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Która kobieta to Twoja siostra?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja muszę iść do pracy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy możesz mi pomóc?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolega chce kupić nową książkę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Myślę, że to dobry pomysł.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy wiesz, gdzie jest moja książka?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muszę dużo pracować, żeby mieć pieniądze.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To jest bardzo ważny dzień w pracy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jestem bardzo zmęczony.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy jesteś dzisiaj zdrowy?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jesteś bardzo dobrym kolegą.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moja babcia jest już stara, ale zdrowa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chcę kupić ten samochód.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wy chcecie pić kawę czy herbatę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja nie mogę teraz iść.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój kolega kupił dzisiaj telefon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Widzę, że masz nowy samochód.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ten mały pies zawsze czeka na mnie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy ten mężczyzna to twój tata?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jutro będę bardzo wesoły!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego ten stary mężczyzna zawsze pije zimną herbatę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiedy Twój kolega chce kupić ten nowy samochód?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy ty słyszysz, co mówi do ciebie mama?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Który pomysł mojego brata lubisz najbardziej?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego wczoraj w nocy byłeś taki smutny?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gdzie mogę kupić dobrą i gorącą kawę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W poniedziałek rano często jestem bardzo zmęczony.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wczoraj dziadek kupił mi bardzo dobrą książkę na urodziny.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Często myślę o tym, co będę robić jutro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dzisiaj jest bardzo ważny dzień dla mojego brata.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wczoraj moja siostra nie chciała iść ze mną do szkoły.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Często nie pamiętam, co mówiłem wczoraj.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dzisiaj nie mogę ci pomóc, bo muszę uczyć się do szkoły.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dziękuję za to, że wczoraj pomogłeś mi w szkole.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zawsze muszę czekać na mojego kolegę po pracy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jestem smutny, że ty nie możesz dzisiaj iść z nami.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bardzo lubię, kiedy mój brat jest taki wesoły.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój brat zawsze chce mieć dużo pieniędzy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wiem, że to jest bardzo ważny czas dla nas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego ten mężczyzna teraz chce pracować w nocy we wtorek?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ile czasu musieliście wczoraj czekać na tatę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Która kobieta we wtorek rano już kupił ten samochód?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gdzie w środę była mama, kiedy wy byliście już w domu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Który to był rok, kiedy dziadek kupił ten stary dom?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy pamiętasz, co w nocy mówił twój przyjaciel?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ile pieniędzy chcesz za ten stary telefon?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tata miał wczoraj dużo pieniędzy, więc kupił mi książkę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On zawsze rano dużo pracuje, ale dzisiaj jest bardzo chory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja dzisiaj nie mam pieniędzy, więc nie mogę kupić tej herbaty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój przyjaciel ma nową pracę, więc dzisiaj jest wesoły.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ta nowa szkoła zawsze uczy, dlaczego czas to pieniądz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój dobry przyjaciel zawsze wie, kiedy ja jestem smutny.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tata mojego kolegi to bardzo dobry i wesoły mężczyzna.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego dziadek nie chce dzisiaj pić ze mną gorącej kawy?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego woda z domu zawsze rano jest taka zimna?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ten duży i stary samochód mojego dziadka jest bardzo dobry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jutro będzie nowy dzień, więc my teraz idziemy już spać.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiedy mam w domu dużo czasu, bardzo lubię dużo myśleć.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zawsze dziękuję za to, że mam dzisiaj gdzie spać</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bardzo dziękuję za to, że twój brat rano uczy mnie migać.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My musimy wiedzieć, dlaczego on wczoraj nie chciał iść.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ten stary mężczyzna bardzo często pije rano dużo gorącej kawy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego ty zawsze dobrze wiesz, gdzie był mój klucz?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kobiety są bardzo zdrowe, bo często dużo pracują w dzień.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Myślałem, że ty wiesz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zostań w poniedziałek u mnie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kupiłem dla ciebie małą książkę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mama często chce pić kawę w nocy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy zawsze jesteś taki smutny przed pracą?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego on nie może pomóc mamie z psem?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wczoraj wieczorem kobieta dziękowała temu mężczyźnie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uczymy się dzisiaj, a jutro idziemy spać.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Twoja mama często robi mi herbatę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ten klucz jest dla mojego kolegi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gdzie mama kupiła tę gorącą kawę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jak dużo pieniędzy może mieć ta kobieta?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kocham pić herbatę z babcią i dziadkiem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Przepraszam, że nie pamiętałem o twoich urodzinach.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy słyszałeś, co mówiła moja siostra?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Musimy pracować w nocy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Musisz dużo jeść, żeby być zdrowym!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy widzieliście, jak on miga?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mam pomysł na nowy dom.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brat często ma dużo czasu dla mamy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ta kobieta czeka na klucz przy szkole.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zawsze w poniedziałek piję zimną wodę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jutro nie mogę pracować, bo jestem bardzo chory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ten rok jest dla nas bardzo dobry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój przyjaciel zawsze rozumie, co mówię.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wczoraj dużo myślałem o tej książce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego twój tata kupił taki stary samochód?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nie lubię, kiedy jesteś bardzo zmęczony po szkole.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To był mój stary telefon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dziękuję ci za ten dobry dzień.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kto ma klucz do domu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mężczyzna czekał na ciebie przed szkołą wczoraj rano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kobiety często piją kawę rano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój mały kot śpi pod starym samochodem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W nocy słyszałem psa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego w poniedziałek pijesz zimną kawę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiedy masz czas na pracę?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ile książek wczoraj kupiłeś?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My lubimy dużo spać w dzień.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Twoja nowa praca jest bardzo ważna.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dziadek i babcia zawsze mają dla mnie czas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja i mój brat chcemy zostać u kolegi na noc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nie chcę pić wody z tobą.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ty zawsze wiesz, gdzie są moje pieniądze!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W poniedziałek rano kupiłem ten samochód dla mamy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiedy ty się uczysz, ja lubię spać.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zawsze myślę, żeby kupić nowy telefon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On czeka w domu na ciebie i na tatę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy twój pies lubi mojego małego kota?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ta zimna noc była dla mnie bardzo smutna.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Widzę cię dzisiaj przed moją pracą.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czego ty wczoraj nie rozumiałeś?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy możemy iść do ciebie wieczorem?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dziadek zawsze pije gorącą herbatę w nocy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kto ci kupił tego psa i kota?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Przepraszam cię za wczoraj.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dlaczego ty zawsze dużo mówisz?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mam bardzo dobry pomysł na jutro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W szkole musimy uczyć się migać.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Twój kolega wczoraj pił ze mną kawę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gdzie są moje pieniądze z poniedziałku?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mój tata bardzo kocha mojego brata.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kobieta przed szkołą kupiła herbatę i kawę.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ty masz czas, żeby ze mną mówić?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jutro zostaniemy w starym domu dziadka.</t>
   </si>
 </sst>
 </file>
@@ -496,19 +946,16 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="238"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="238"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -553,7 +1000,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -566,11 +1013,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -697,8 +1140,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D301"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46.32"/>
@@ -715,7 +1158,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -729,7 +1172,7 @@
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -740,10 +1183,10 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -754,10 +1197,10 @@
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -768,10 +1211,10 @@
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -782,10 +1225,10 @@
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -796,10 +1239,10 @@
       <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -810,10 +1253,10 @@
       <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -824,10 +1267,10 @@
       <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -838,10 +1281,10 @@
       <c r="B10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -852,10 +1295,10 @@
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -866,10 +1309,10 @@
       <c r="B12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -880,10 +1323,10 @@
       <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -894,10 +1337,10 @@
       <c r="B14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -908,10 +1351,10 @@
       <c r="B15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -922,10 +1365,10 @@
       <c r="B16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -936,10 +1379,10 @@
       <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -950,10 +1393,10 @@
       <c r="B18" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -964,10 +1407,10 @@
       <c r="B19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -978,10 +1421,10 @@
       <c r="B20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -992,10 +1435,10 @@
       <c r="B21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1006,10 +1449,10 @@
       <c r="B22" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1020,10 +1463,10 @@
       <c r="B23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1034,10 +1477,10 @@
       <c r="B24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1048,10 +1491,10 @@
       <c r="B25" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1062,10 +1505,10 @@
       <c r="B26" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1076,10 +1519,10 @@
       <c r="B27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1087,10 +1530,10 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1098,10 +1541,10 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1112,10 +1555,10 @@
       <c r="B30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1126,10 +1569,10 @@
       <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1140,10 +1583,10 @@
       <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1154,10 +1597,10 @@
       <c r="B33" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1168,10 +1611,10 @@
       <c r="B34" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D34" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1182,10 +1625,10 @@
       <c r="B35" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D35" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1196,10 +1639,10 @@
       <c r="B36" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D36" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1210,10 +1653,10 @@
       <c r="B37" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1224,10 +1667,10 @@
       <c r="B38" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D38" s="3" t="n">
+      <c r="D38" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1238,10 +1681,10 @@
       <c r="B39" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1252,10 +1695,10 @@
       <c r="B40" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D40" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1266,10 +1709,10 @@
       <c r="B41" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1280,10 +1723,10 @@
       <c r="B42" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D42" s="3" t="n">
+      <c r="D42" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1294,10 +1737,10 @@
       <c r="B43" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D43" s="3" t="n">
+      <c r="D43" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1308,10 +1751,10 @@
       <c r="B44" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D44" s="3" t="n">
+      <c r="D44" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1322,10 +1765,10 @@
       <c r="B45" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D45" s="3" t="n">
+      <c r="D45" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1336,10 +1779,10 @@
       <c r="B46" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D46" s="3" t="n">
+      <c r="D46" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1350,10 +1793,10 @@
       <c r="B47" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D47" s="3" t="n">
+      <c r="D47" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1364,10 +1807,10 @@
       <c r="B48" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D48" s="3" t="n">
+      <c r="D48" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1378,10 +1821,10 @@
       <c r="B49" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D49" s="3" t="n">
+      <c r="D49" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1392,10 +1835,10 @@
       <c r="B50" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D50" s="3" t="n">
+      <c r="D50" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1406,10 +1849,10 @@
       <c r="B51" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D51" s="3" t="n">
+      <c r="D51" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1417,10 +1860,10 @@
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="0" t="s">
+      <c r="B52" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D52" s="3" t="n">
+      <c r="D52" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1428,10 +1871,10 @@
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="0" t="s">
+      <c r="B53" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D53" s="3" t="n">
+      <c r="D53" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1439,10 +1882,10 @@
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="0" t="s">
+      <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D54" s="3" t="n">
+      <c r="D54" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1450,10 +1893,10 @@
       <c r="A55" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="0" t="s">
+      <c r="B55" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D55" s="3" t="n">
+      <c r="D55" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1461,10 +1904,10 @@
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="0" t="s">
+      <c r="B56" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D56" s="3" t="n">
+      <c r="D56" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1472,10 +1915,10 @@
       <c r="A57" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="0" t="s">
+      <c r="B57" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D57" s="3" t="n">
+      <c r="D57" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1483,10 +1926,10 @@
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="0" t="s">
+      <c r="B58" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="D58" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1494,10 +1937,10 @@
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="0" t="s">
+      <c r="B59" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D59" s="3" t="n">
+      <c r="D59" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1505,10 +1948,10 @@
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="0" t="s">
+      <c r="B60" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D60" s="3" t="n">
+      <c r="D60" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1516,10 +1959,10 @@
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="0" t="s">
+      <c r="B61" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D61" s="3" t="n">
+      <c r="D61" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1527,10 +1970,10 @@
       <c r="A62" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="0" t="s">
+      <c r="B62" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D62" s="3" t="n">
+      <c r="D62" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1538,10 +1981,10 @@
       <c r="A63" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="0" t="s">
+      <c r="B63" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D63" s="3" t="n">
+      <c r="D63" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1549,10 +1992,10 @@
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="0" t="s">
+      <c r="B64" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D64" s="3" t="n">
+      <c r="D64" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1560,10 +2003,10 @@
       <c r="A65" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="0" t="s">
+      <c r="B65" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D65" s="3" t="n">
+      <c r="D65" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1571,10 +2014,10 @@
       <c r="A66" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="0" t="s">
+      <c r="B66" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D66" s="3" t="n">
+      <c r="D66" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1582,10 +2025,10 @@
       <c r="A67" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="0" t="s">
+      <c r="B67" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D67" s="3" t="n">
+      <c r="D67" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1593,10 +2036,10 @@
       <c r="A68" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="0" t="s">
+      <c r="B68" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D68" s="3" t="n">
+      <c r="D68" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1604,10 +2047,10 @@
       <c r="A69" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="0" t="s">
+      <c r="B69" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D69" s="3" t="n">
+      <c r="D69" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1615,10 +2058,10 @@
       <c r="A70" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="0" t="s">
+      <c r="B70" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D70" s="3" t="n">
+      <c r="D70" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1626,10 +2069,10 @@
       <c r="A71" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="0" t="s">
+      <c r="B71" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D71" s="3" t="n">
+      <c r="D71" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1637,10 +2080,10 @@
       <c r="A72" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="0" t="s">
+      <c r="B72" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D72" s="3" t="n">
+      <c r="D72" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1648,10 +2091,10 @@
       <c r="A73" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="0" t="s">
+      <c r="B73" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D73" s="3" t="n">
+      <c r="D73" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1659,10 +2102,10 @@
       <c r="A74" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="0" t="s">
+      <c r="B74" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D74" s="3" t="n">
+      <c r="D74" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1670,10 +2113,10 @@
       <c r="A75" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="0" t="s">
+      <c r="B75" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D75" s="3" t="n">
+      <c r="D75" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1681,10 +2124,10 @@
       <c r="A76" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="0" t="s">
+      <c r="B76" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D76" s="3" t="n">
+      <c r="D76" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1692,10 +2135,10 @@
       <c r="A77" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="0" t="s">
+      <c r="B77" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D77" s="3" t="n">
+      <c r="D77" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1703,10 +2146,10 @@
       <c r="A78" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="0" t="s">
+      <c r="B78" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D78" s="3" t="n">
+      <c r="D78" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1714,10 +2157,10 @@
       <c r="A79" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="0" t="s">
+      <c r="B79" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D79" s="3" t="n">
+      <c r="D79" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1725,10 +2168,10 @@
       <c r="A80" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="0" t="s">
+      <c r="B80" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D80" s="3" t="n">
+      <c r="D80" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1736,10 +2179,10 @@
       <c r="A81" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="B81" s="0" t="s">
+      <c r="B81" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D81" s="3" t="n">
+      <c r="D81" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1747,10 +2190,10 @@
       <c r="A82" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="B82" s="0" t="s">
+      <c r="B82" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D82" s="3" t="n">
+      <c r="D82" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1758,10 +2201,10 @@
       <c r="A83" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="B83" s="0" t="s">
+      <c r="B83" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D83" s="3" t="n">
+      <c r="D83" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1769,10 +2212,10 @@
       <c r="A84" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="B84" s="0" t="s">
+      <c r="B84" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D84" s="3" t="n">
+      <c r="D84" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1780,10 +2223,10 @@
       <c r="A85" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="B85" s="0" t="s">
+      <c r="B85" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D85" s="3" t="n">
+      <c r="D85" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1791,10 +2234,10 @@
       <c r="A86" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="B86" s="0" t="s">
+      <c r="B86" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D86" s="3" t="n">
+      <c r="D86" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1802,10 +2245,10 @@
       <c r="A87" s="2" t="n">
         <v>86</v>
       </c>
-      <c r="B87" s="0" t="s">
+      <c r="B87" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D87" s="3" t="n">
+      <c r="D87" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1813,10 +2256,10 @@
       <c r="A88" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="B88" s="0" t="s">
+      <c r="B88" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D88" s="3" t="n">
+      <c r="D88" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1824,10 +2267,10 @@
       <c r="A89" s="2" t="n">
         <v>88</v>
       </c>
-      <c r="B89" s="0" t="s">
+      <c r="B89" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D89" s="3" t="n">
+      <c r="D89" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1835,10 +2278,10 @@
       <c r="A90" s="2" t="n">
         <v>89</v>
       </c>
-      <c r="B90" s="0" t="s">
+      <c r="B90" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D90" s="3" t="n">
+      <c r="D90" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1846,10 +2289,10 @@
       <c r="A91" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="B91" s="0" t="s">
+      <c r="B91" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D91" s="3" t="n">
+      <c r="D91" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1857,10 +2300,10 @@
       <c r="A92" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="B92" s="0" t="s">
+      <c r="B92" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D92" s="3" t="n">
+      <c r="D92" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1868,10 +2311,10 @@
       <c r="A93" s="2" t="n">
         <v>92</v>
       </c>
-      <c r="B93" s="0" t="s">
+      <c r="B93" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D93" s="3" t="n">
+      <c r="D93" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1879,10 +2322,10 @@
       <c r="A94" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="B94" s="0" t="s">
+      <c r="B94" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D94" s="3" t="n">
+      <c r="D94" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1890,10 +2333,10 @@
       <c r="A95" s="2" t="n">
         <v>94</v>
       </c>
-      <c r="B95" s="0" t="s">
+      <c r="B95" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D95" s="3" t="n">
+      <c r="D95" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1901,10 +2344,10 @@
       <c r="A96" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="B96" s="0" t="s">
+      <c r="B96" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D96" s="3" t="n">
+      <c r="D96" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1912,10 +2355,10 @@
       <c r="A97" s="2" t="n">
         <v>96</v>
       </c>
-      <c r="B97" s="0" t="s">
+      <c r="B97" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D97" s="3" t="n">
+      <c r="D97" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1923,10 +2366,10 @@
       <c r="A98" s="2" t="n">
         <v>97</v>
       </c>
-      <c r="B98" s="0" t="s">
+      <c r="B98" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="D98" s="3" t="n">
+      <c r="D98" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1934,10 +2377,10 @@
       <c r="A99" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="B99" s="0" t="s">
+      <c r="B99" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D99" s="3" t="n">
+      <c r="D99" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1945,10 +2388,10 @@
       <c r="A100" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="B100" s="0" t="s">
+      <c r="B100" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D100" s="3" t="n">
+      <c r="D100" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1956,20 +2399,1820 @@
       <c r="A101" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="B101" s="0" t="s">
+      <c r="B101" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D101" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="D101" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="D104" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="D105" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="D106" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D110" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="D111" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="D112" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="D113" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="D114" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="D117" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="D118" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D119" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="D120" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="D122" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="2" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="D129" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="D131" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="D132" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="D133" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="D134" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="D135" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="D136" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="D137" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="D138" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="D139" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="0" t="s">
+        <v>190</v>
+      </c>
+      <c r="D140" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="D141" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="D142" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="D144" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="D145" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="D146" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="D147" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="D148" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="2" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="D149" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="D150" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="D151" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="2" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="D153" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="D154" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="2" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="D155" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="D156" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="D159" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="2" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="0" t="s">
+        <v>210</v>
+      </c>
+      <c r="D160" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="D161" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="2" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="D162" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="2" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="D163" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="D164" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="2" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="D165" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="2" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="D166" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="2" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="D167" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="2" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="D168" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" s="0" t="s">
+        <v>219</v>
+      </c>
+      <c r="D169" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="D170" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="D171" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="D172" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="D173" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="2" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="D174" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="2" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="D175" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="D176" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="D177" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="D178" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="D179" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="2" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="D180" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="D181" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="D182" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="D183" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="2" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="D184" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="2" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="D185" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="D186" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="D187" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="D188" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="D189" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="2" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="0" t="s">
+        <v>240</v>
+      </c>
+      <c r="D190" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="D191" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="0" t="s">
+        <v>242</v>
+      </c>
+      <c r="D192" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="D193" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="2" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="D194" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="2" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="D195" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="2" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="D196" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="2" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="D197" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="2" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="D198" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="D199" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="2" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" s="0" t="s">
+        <v>250</v>
+      </c>
+      <c r="D200" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="D201" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="D202" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="D203" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="2" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="D204" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="2" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="D205" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="2" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="D206" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="2" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="D207" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="2" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="D208" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="D209" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="2" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="D210" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="D211" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="2" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="D212" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="2" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="D213" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="2" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="D214" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="2" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="D215" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="D216" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="2" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="D217" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="2" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="D218" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="D219" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="2" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="D220" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="D221" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="2" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="D222" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="2" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" s="0" t="s">
+        <v>273</v>
+      </c>
+      <c r="D223" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="D224" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="2" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="D225" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="2" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" s="0" t="s">
+        <v>276</v>
+      </c>
+      <c r="D226" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" s="0" t="s">
+        <v>277</v>
+      </c>
+      <c r="D227" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="2" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="D228" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="D229" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="2" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="D230" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="0" t="s">
+        <v>281</v>
+      </c>
+      <c r="D231" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="0" t="s">
+        <v>282</v>
+      </c>
+      <c r="D232" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="2" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" s="0" t="s">
+        <v>283</v>
+      </c>
+      <c r="D233" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="2" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" s="0" t="s">
+        <v>284</v>
+      </c>
+      <c r="D234" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="2" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="0" t="s">
+        <v>285</v>
+      </c>
+      <c r="D235" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="2" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="0" t="s">
+        <v>286</v>
+      </c>
+      <c r="D236" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="2" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" s="0" t="s">
+        <v>287</v>
+      </c>
+      <c r="D237" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="2" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="D238" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="2" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" s="0" t="s">
+        <v>289</v>
+      </c>
+      <c r="D239" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="2" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="0" t="s">
+        <v>290</v>
+      </c>
+      <c r="D240" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="0" t="s">
+        <v>291</v>
+      </c>
+      <c r="D241" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="2" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" s="0" t="s">
+        <v>292</v>
+      </c>
+      <c r="D242" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="2" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="D243" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="2" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" s="0" t="s">
+        <v>294</v>
+      </c>
+      <c r="D244" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="2" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" s="0" t="s">
+        <v>295</v>
+      </c>
+      <c r="D245" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="2" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" s="0" t="s">
+        <v>296</v>
+      </c>
+      <c r="D246" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="2" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" s="0" t="s">
+        <v>297</v>
+      </c>
+      <c r="D247" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="2" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="D248" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="2" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" s="0" t="s">
+        <v>299</v>
+      </c>
+      <c r="D249" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" s="0" t="s">
+        <v>300</v>
+      </c>
+      <c r="D250" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" s="0" t="s">
+        <v>301</v>
+      </c>
+      <c r="D251" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D252" s="2"/>
+    </row>
+    <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D253" s="2"/>
+    </row>
+    <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D254" s="2"/>
+    </row>
+    <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D255" s="2"/>
+    </row>
+    <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D256" s="2"/>
+    </row>
+    <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D257" s="2"/>
+    </row>
+    <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D258" s="2"/>
+    </row>
+    <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D259" s="2"/>
+    </row>
+    <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D260" s="2"/>
+    </row>
+    <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D261" s="2"/>
+    </row>
+    <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D262" s="2"/>
+    </row>
+    <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D263" s="2"/>
+    </row>
+    <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D264" s="2"/>
+    </row>
+    <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D265" s="2"/>
+    </row>
+    <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D266" s="2"/>
+    </row>
+    <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D267" s="2"/>
+    </row>
+    <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D268" s="2"/>
+    </row>
+    <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D269" s="2"/>
+    </row>
+    <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D270" s="2"/>
+    </row>
+    <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D271" s="2"/>
+    </row>
+    <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D272" s="2"/>
+    </row>
+    <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D273" s="2"/>
+    </row>
+    <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D274" s="2"/>
+    </row>
+    <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D275" s="2"/>
+    </row>
+    <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D276" s="2"/>
+    </row>
+    <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D277" s="2"/>
+    </row>
+    <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D278" s="2"/>
+    </row>
+    <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D279" s="2"/>
+    </row>
+    <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D280" s="2"/>
+    </row>
+    <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D281" s="2"/>
+    </row>
+    <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D282" s="2"/>
+    </row>
+    <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D283" s="2"/>
+    </row>
+    <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D284" s="2"/>
+    </row>
+    <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D285" s="2"/>
+    </row>
+    <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D286" s="2"/>
+    </row>
+    <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D287" s="2"/>
+    </row>
+    <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D288" s="2"/>
+    </row>
+    <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D289" s="2"/>
+    </row>
+    <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D290" s="2"/>
+    </row>
+    <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D291" s="2"/>
+    </row>
+    <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D292" s="2"/>
+    </row>
+    <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D293" s="2"/>
+    </row>
+    <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D294" s="2"/>
+    </row>
+    <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D295" s="2"/>
+    </row>
+    <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D296" s="2"/>
+    </row>
+    <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D297" s="2"/>
+    </row>
+    <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D298" s="2"/>
+    </row>
+    <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D299" s="2"/>
+    </row>
+    <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D300" s="2"/>
+    </row>
+    <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D301" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normalny"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normalny"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added analysis sentences app
</commit_message>
<xml_diff>
--- a/Sentences/prepared_sentences.xlsx
+++ b/Sentences/prepared_sentences.xlsx
@@ -739,7 +739,7 @@
     <t xml:space="preserve">Co robisz rano?</t>
   </si>
   <si>
-    <t xml:space="preserve">TY, RANO, CO, ROBIĆ</t>
+    <t xml:space="preserve">TY, RANO, ROBIĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Gdzie jest twój telefon?</t>
@@ -781,7 +781,7 @@
     <t xml:space="preserve">Myślę, że to dobry pomysł.</t>
   </si>
   <si>
-    <t xml:space="preserve">JA, MYŚLEĆ, TO, POMYSŁ, DOBRY</t>
+    <t xml:space="preserve">JA, MYŚLEĆ, POMYSŁ, DOBRY</t>
   </si>
   <si>
     <t xml:space="preserve">Czy wiesz, gdzie jest moja książka?</t>
@@ -799,7 +799,7 @@
     <t xml:space="preserve">To jest bardzo ważny dzień w pracy.</t>
   </si>
   <si>
-    <t xml:space="preserve">TO, DZIEŃ, BARDZO, WAŻNY, PRACA</t>
+    <t xml:space="preserve">DZIEŃ, BARDZO, WAŻNY, PRACA</t>
   </si>
   <si>
     <t xml:space="preserve">Jestem bardzo zmęczony.</t>
@@ -1027,7 +1027,7 @@
     <t xml:space="preserve">Ile pieniędzy chcesz za ten stary telefon?</t>
   </si>
   <si>
-    <t xml:space="preserve">TY, CHCIEĆ, ILE, PIENIĄDZE, TELEFON, STARY, TEN</t>
+    <t xml:space="preserve">TY, CHCIEĆ, ILE, PIENIĄDZE, TELEFON, STARY</t>
   </si>
   <si>
     <t xml:space="preserve">Tata miał wczoraj dużo pieniędzy, więc kupił mi książkę.</t>
@@ -1045,19 +1045,19 @@
     <t xml:space="preserve">Ja dzisiaj nie mam pieniędzy, więc nie mogę kupić tej herbaty.</t>
   </si>
   <si>
-    <t xml:space="preserve">DZISIAJ, JA, PIENIĄDZE, NIE-MIEĆ, WIĘC, HERBATA, TA, KUPIĆ, NIE-MÓC</t>
+    <t xml:space="preserve">DZISIAJ, JA, PIENIĄDZE, NIE-MIEĆ, HERBATA, KUPIĆ, NIE-MÓC</t>
   </si>
   <si>
     <t xml:space="preserve">Mój przyjaciel ma nową pracę, więc dzisiaj jest wesoły.</t>
   </si>
   <si>
-    <t xml:space="preserve">MÓJ, PRZYJACIEL, PRACA, NOWA, MIEĆ, WIĘC, DZISIAJ, WESOŁY</t>
+    <t xml:space="preserve">MÓJ, PRZYJACIEL, PRACA, NOWA, MIEĆ, DZISIAJ, WESOŁY</t>
   </si>
   <si>
     <t xml:space="preserve">Ta nowa szkoła zawsze uczy, dlaczego czas to pieniądz.</t>
   </si>
   <si>
-    <t xml:space="preserve">SZKOŁA, NOWA, TA, ZAWSZE, UCZYĆ, DLACZEGO, CZAS, PIENIĄDZ</t>
+    <t xml:space="preserve">SZKOŁA, NOWA, ZAWSZE, UCZYĆ, DLACZEGO, CZAS, PIENIĄDZ</t>
   </si>
   <si>
     <t xml:space="preserve">Mój dobry przyjaciel zawsze wie, kiedy ja jestem smutny.</t>
@@ -1093,7 +1093,7 @@
     <t xml:space="preserve">Jutro będzie nowy dzień, więc my teraz idziemy już spać.</t>
   </si>
   <si>
-    <t xml:space="preserve">JUTRO, DZIEŃ, NOWY, WIĘC, TERAZ, MY, SPAĆ, IŚĆ</t>
+    <t xml:space="preserve">JUTRO, DZIEŃ, NOWY, TERAZ, MY, SPAĆ, IŚĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Kiedy mam w domu dużo czasu, bardzo lubię dużo myśleć.</t>
@@ -1177,7 +1177,7 @@
     <t xml:space="preserve">Wczoraj wieczorem kobieta dziękowała temu mężczyźnie.</t>
   </si>
   <si>
-    <t xml:space="preserve">WCZORAJ, WIECZÓR, KOBIETA, MĘŻCZYZNA, TEMU, DZIĘKOWAĆ</t>
+    <t xml:space="preserve">WCZORAJ, WIECZÓR, KOBIETA, MĘŻCZYZNA, DZIĘKOWAĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Uczymy się dzisiaj, a jutro idziemy spać.</t>
@@ -1201,19 +1201,19 @@
     <t xml:space="preserve">Gdzie mama kupiła tę gorącą kawę?</t>
   </si>
   <si>
-    <t xml:space="preserve">MAMA, GDZIE, KAWA, GORĄCA, TA, KUPIĆ</t>
+    <t xml:space="preserve">MAMA, GDZIE, KAWA, GORĄCA, KUPIĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Jak dużo pieniędzy może mieć ta kobieta?</t>
   </si>
   <si>
-    <t xml:space="preserve">KOBIETA, TA, PIENIĄDZE, ILE, MIEĆ, MOŻE</t>
+    <t xml:space="preserve">KOBIETA, PIENIĄDZE, ILE, MIEĆ, MOŻE</t>
   </si>
   <si>
     <t xml:space="preserve">Kocham pić herbatę z babcią i dziadkiem.</t>
   </si>
   <si>
-    <t xml:space="preserve">JA, KOCHAĆ, HERBATA, PIĆ, BABCIA, DZIADEK, Z</t>
+    <t xml:space="preserve">JA, KOCHAĆ, HERBATA, PIĆ, BABCIA, DZIADEK</t>
   </si>
   <si>
     <t xml:space="preserve">Przepraszam, że nie pamiętałem o twoich urodzinach.</t>
@@ -1237,7 +1237,7 @@
     <t xml:space="preserve">Musisz dużo jeść, żeby być zdrowym!</t>
   </si>
   <si>
-    <t xml:space="preserve">TY, MUSIEĆ, JEŚĆ, DUŻO, ZDROWY, BYĆ</t>
+    <t xml:space="preserve">TY, MUSIEĆ, JEŚĆ, DUŻO, ZDROWY</t>
   </si>
   <si>
     <t xml:space="preserve">Czy widzieliście, jak on miga?</t>
@@ -1255,13 +1255,13 @@
     <t xml:space="preserve">Brat często ma dużo czasu dla mamy.</t>
   </si>
   <si>
-    <t xml:space="preserve">BRAT, CZĘSTO, CZAS, DUŻO, MAMA, DLA, MIEĆ</t>
+    <t xml:space="preserve">BRAT, CZĘSTO, CZAS, DUŻO, DLA, MAMA</t>
   </si>
   <si>
     <t xml:space="preserve">Ta kobieta czeka na klucz przy szkole.</t>
   </si>
   <si>
-    <t xml:space="preserve">KOBIETA, TA, SZKOŁA, PRZY, KLUCZ, CZEKAĆ</t>
+    <t xml:space="preserve">KOBIETA, SZKOŁA, KLUCZ, CZEKAĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Zawsze w poniedziałek piję zimną wodę.</t>
@@ -1273,13 +1273,13 @@
     <t xml:space="preserve">Jutro nie mogę pracować, bo jestem bardzo chory.</t>
   </si>
   <si>
-    <t xml:space="preserve">JUTRO, JA, PRACOWAĆ, NIE-MÓC, BO, JA, BARDZO, CHORY</t>
+    <t xml:space="preserve">JUTRO, JA, PRACOWAĆ, NIE-MÓC, JA, BARDZO, CHORY</t>
   </si>
   <si>
     <t xml:space="preserve">Ten rok jest dla nas bardzo dobry.</t>
   </si>
   <si>
-    <t xml:space="preserve">ROK, TEN, DLA-NAS, BARDZO, DOBRY</t>
+    <t xml:space="preserve">ROK, DLA-NAS, BARDZO, DOBRY</t>
   </si>
   <si>
     <t xml:space="preserve">Mój przyjaciel zawsze rozumie, co mówię.</t>
@@ -1291,13 +1291,13 @@
     <t xml:space="preserve">Wczoraj dużo myślałem o tej książce.</t>
   </si>
   <si>
-    <t xml:space="preserve">WCZORAJ, JA, MYŚLEĆ, DUŻO, KSIĄŻKA, TA</t>
+    <t xml:space="preserve">WCZORAJ, JA, MYŚLEĆ, DUŻO, TA, KSIĄŻKA</t>
   </si>
   <si>
     <t xml:space="preserve">Dlaczego twój tata kupił taki stary samochód?</t>
   </si>
   <si>
-    <t xml:space="preserve">TWÓJ, TATA, DLACZEGO, SAMOCHÓD, STARY, TAKI, KUPIĆ</t>
+    <t xml:space="preserve">TWÓJ, TATA, DLACZEGO, SAMOCHÓD, STARY, KUPIĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Nie lubię, kiedy jesteś bardzo zmęczony po szkole.</t>
@@ -1309,19 +1309,19 @@
     <t xml:space="preserve">To był mój stary telefon.</t>
   </si>
   <si>
-    <t xml:space="preserve">TO, MÓJ, TELEFON, STARY, BYĆ</t>
+    <t xml:space="preserve">MÓJ, TELEFON, STARY, BYĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Dziękuję ci za ten dobry dzień.</t>
   </si>
   <si>
-    <t xml:space="preserve">DZIĘKUJĘ, CI, DZIEŃ, DOBRY, TEN</t>
+    <t xml:space="preserve">DZIĘKUJĘ, CI, DZIEŃ, DOBRY</t>
   </si>
   <si>
     <t xml:space="preserve">Kto ma klucz do domu?</t>
   </si>
   <si>
-    <t xml:space="preserve">KTO, KLUCZ, DOM, DO, MIEĆ</t>
+    <t xml:space="preserve">KTO, KLUCZ, DOM, MIEĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Mężczyzna czekał na ciebie przed szkołą wczoraj rano.</t>
@@ -1357,7 +1357,7 @@
     <t xml:space="preserve">Kiedy masz czas na pracę?</t>
   </si>
   <si>
-    <t xml:space="preserve">TY, KIEDY, CZAS, PRACA, NA, MIEĆ</t>
+    <t xml:space="preserve">TY, KIEDY, CZAS, PRACA, MIEĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Ile książek wczoraj kupiłeś?</t>
@@ -1381,7 +1381,7 @@
     <t xml:space="preserve">Dziadek i babcia zawsze mają dla mnie czas.</t>
   </si>
   <si>
-    <t xml:space="preserve">DZIADEK+BABCIA, ZAWSZE, MI, CZAS, MIEĆ</t>
+    <t xml:space="preserve">DZIADEK+BABCIA, ZAWSZE, MI, CZAS</t>
   </si>
   <si>
     <t xml:space="preserve">Ja i mój brat chcemy zostać u kolegi na noc.</t>
@@ -1423,7 +1423,7 @@
     <t xml:space="preserve">On czeka w domu na ciebie i na tatę.</t>
   </si>
   <si>
-    <t xml:space="preserve">ON, DOM, NA-CIEBIE, I, TATA, CZEKAĆ</t>
+    <t xml:space="preserve">ON, DOM, NA-CIEBIE, TATA, CZEKAĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Czy twój pies lubi mojego małego kota?</t>
@@ -1435,7 +1435,7 @@
     <t xml:space="preserve">Ta zimna noc była dla mnie bardzo smutna.</t>
   </si>
   <si>
-    <t xml:space="preserve">NOC, ZIMNA, TA, DLA-MNIE, BARDZO, SMUTNA</t>
+    <t xml:space="preserve">NOC, ZIMNA, DLA-MNIE, BARDZO, SMUTNA</t>
   </si>
   <si>
     <t xml:space="preserve">Widzę cię dzisiaj przed moją pracą.</t>
@@ -1453,7 +1453,7 @@
     <t xml:space="preserve">Czy możemy iść do ciebie wieczorem?</t>
   </si>
   <si>
-    <t xml:space="preserve">MY, WIECZÓR, DO-CIEBIE, IŚĆ, MOŻNA</t>
+    <t xml:space="preserve">MY, WIECZÓR, DO-CIEBIE, MOŻNA</t>
   </si>
   <si>
     <t xml:space="preserve">Dziadek zawsze pije gorącą herbatę w nocy.</t>
@@ -1465,7 +1465,7 @@
     <t xml:space="preserve">Kto ci kupił tego psa i kota?</t>
   </si>
   <si>
-    <t xml:space="preserve">KTO, CI, PIES, TEN, I, KOT, KUPIĆ</t>
+    <t xml:space="preserve">KTO, CI, PIES, TEN, KOT, KUPIĆ</t>
   </si>
   <si>
     <t xml:space="preserve">Przepraszam cię za wczoraj.</t>
@@ -1483,7 +1483,7 @@
     <t xml:space="preserve">Mam bardzo dobry pomysł na jutro.</t>
   </si>
   <si>
-    <t xml:space="preserve">JA, POMYSŁ, BARDZO, DOBRY, JUTRO, NA, MIEĆ</t>
+    <t xml:space="preserve">JA, MIEĆ, POMYSŁ, BARDZO, DOBRY, JUTRO </t>
   </si>
   <si>
     <t xml:space="preserve">W szkole musimy uczyć się migać.</t>
@@ -1501,7 +1501,7 @@
     <t xml:space="preserve">Gdzie są moje pieniądze z poniedziałku?</t>
   </si>
   <si>
-    <t xml:space="preserve">MOJE, PIENIĄDZE, PONIEDZIAŁEK, Z, GDZIE</t>
+    <t xml:space="preserve">MOJE, PIENIĄDZE, PONIEDZIAŁEK, GDZIE</t>
   </si>
   <si>
     <t xml:space="preserve">Mój tata bardzo kocha mojego brata.</t>
@@ -1600,7 +1600,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1614,10 +1614,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2467,7 +2463,7 @@
       <c r="B52" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="3" t="s">
         <v>103</v>
       </c>
       <c r="D52" s="2" t="n">
@@ -2481,7 +2477,7 @@
       <c r="B53" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="3" t="s">
         <v>105</v>
       </c>
       <c r="D53" s="2" t="n">
@@ -2495,7 +2491,7 @@
       <c r="B54" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C54" s="3" t="s">
         <v>107</v>
       </c>
       <c r="D54" s="2" t="n">
@@ -2509,7 +2505,7 @@
       <c r="B55" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="3" t="s">
         <v>109</v>
       </c>
       <c r="D55" s="2" t="n">
@@ -2523,7 +2519,7 @@
       <c r="B56" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="3" t="s">
         <v>111</v>
       </c>
       <c r="D56" s="2" t="n">
@@ -2537,7 +2533,7 @@
       <c r="B57" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C57" s="3" t="s">
         <v>113</v>
       </c>
       <c r="D57" s="2" t="n">
@@ -2551,7 +2547,7 @@
       <c r="B58" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="C58" s="3" t="s">
         <v>115</v>
       </c>
       <c r="D58" s="2" t="n">
@@ -2565,7 +2561,7 @@
       <c r="B59" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="3" t="s">
         <v>117</v>
       </c>
       <c r="D59" s="2" t="n">
@@ -2579,7 +2575,7 @@
       <c r="B60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="3" t="s">
         <v>119</v>
       </c>
       <c r="D60" s="2" t="n">
@@ -2593,7 +2589,7 @@
       <c r="B61" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="3" t="s">
         <v>121</v>
       </c>
       <c r="D61" s="2" t="n">
@@ -2607,7 +2603,7 @@
       <c r="B62" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="C62" s="3" t="s">
         <v>123</v>
       </c>
       <c r="D62" s="2" t="n">
@@ -2621,7 +2617,7 @@
       <c r="B63" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C63" s="4" t="s">
+      <c r="C63" s="3" t="s">
         <v>125</v>
       </c>
       <c r="D63" s="2" t="n">
@@ -2635,7 +2631,7 @@
       <c r="B64" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="C64" s="3" t="s">
         <v>127</v>
       </c>
       <c r="D64" s="2" t="n">
@@ -2649,7 +2645,7 @@
       <c r="B65" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="C65" s="3" t="s">
         <v>129</v>
       </c>
       <c r="D65" s="2" t="n">
@@ -2663,7 +2659,7 @@
       <c r="B66" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C66" s="4" t="s">
+      <c r="C66" s="3" t="s">
         <v>131</v>
       </c>
       <c r="D66" s="2" t="n">
@@ -2677,7 +2673,7 @@
       <c r="B67" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C67" s="4" t="s">
+      <c r="C67" s="3" t="s">
         <v>133</v>
       </c>
       <c r="D67" s="2" t="n">
@@ -2691,7 +2687,7 @@
       <c r="B68" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="3" t="s">
         <v>135</v>
       </c>
       <c r="D68" s="2" t="n">
@@ -2705,7 +2701,7 @@
       <c r="B69" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C69" s="4" t="s">
+      <c r="C69" s="3" t="s">
         <v>137</v>
       </c>
       <c r="D69" s="2" t="n">
@@ -2719,7 +2715,7 @@
       <c r="B70" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C70" s="4" t="s">
+      <c r="C70" s="3" t="s">
         <v>139</v>
       </c>
       <c r="D70" s="2" t="n">
@@ -2733,7 +2729,7 @@
       <c r="B71" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C71" s="4" t="s">
+      <c r="C71" s="3" t="s">
         <v>141</v>
       </c>
       <c r="D71" s="2" t="n">
@@ -2747,7 +2743,7 @@
       <c r="B72" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="C72" s="3" t="s">
         <v>143</v>
       </c>
       <c r="D72" s="2" t="n">
@@ -2761,7 +2757,7 @@
       <c r="B73" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="C73" s="4" t="s">
+      <c r="C73" s="3" t="s">
         <v>145</v>
       </c>
       <c r="D73" s="2" t="n">
@@ -2775,7 +2771,7 @@
       <c r="B74" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C74" s="4" t="s">
+      <c r="C74" s="3" t="s">
         <v>147</v>
       </c>
       <c r="D74" s="2" t="n">
@@ -2789,7 +2785,7 @@
       <c r="B75" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="C75" s="3" t="s">
         <v>149</v>
       </c>
       <c r="D75" s="2" t="n">
@@ -2803,7 +2799,7 @@
       <c r="B76" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="C76" s="3" t="s">
         <v>151</v>
       </c>
       <c r="D76" s="2" t="n">
@@ -2817,7 +2813,7 @@
       <c r="B77" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C77" s="3" t="s">
         <v>153</v>
       </c>
       <c r="D77" s="2" t="n">
@@ -2831,7 +2827,7 @@
       <c r="B78" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C78" s="3" t="s">
         <v>155</v>
       </c>
       <c r="D78" s="2" t="n">
@@ -2845,7 +2841,7 @@
       <c r="B79" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="C79" s="3" t="s">
         <v>157</v>
       </c>
       <c r="D79" s="2" t="n">
@@ -2859,7 +2855,7 @@
       <c r="B80" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C80" s="4" t="s">
+      <c r="C80" s="3" t="s">
         <v>159</v>
       </c>
       <c r="D80" s="2" t="n">
@@ -2873,7 +2869,7 @@
       <c r="B81" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="3" t="s">
         <v>161</v>
       </c>
       <c r="D81" s="2" t="n">
@@ -2887,7 +2883,7 @@
       <c r="B82" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="C82" s="3" t="s">
         <v>163</v>
       </c>
       <c r="D82" s="2" t="n">
@@ -2901,7 +2897,7 @@
       <c r="B83" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="4" t="s">
+      <c r="C83" s="3" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="2" t="n">
@@ -2915,7 +2911,7 @@
       <c r="B84" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="3" t="s">
         <v>167</v>
       </c>
       <c r="D84" s="2" t="n">
@@ -2929,7 +2925,7 @@
       <c r="B85" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C85" s="4" t="s">
+      <c r="C85" s="3" t="s">
         <v>169</v>
       </c>
       <c r="D85" s="2" t="n">
@@ -2943,7 +2939,7 @@
       <c r="B86" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C86" s="4" t="s">
+      <c r="C86" s="3" t="s">
         <v>171</v>
       </c>
       <c r="D86" s="2" t="n">
@@ -2957,7 +2953,7 @@
       <c r="B87" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C87" s="3" t="s">
         <v>173</v>
       </c>
       <c r="D87" s="2" t="n">
@@ -2971,7 +2967,7 @@
       <c r="B88" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C88" s="4" t="s">
+      <c r="C88" s="3" t="s">
         <v>175</v>
       </c>
       <c r="D88" s="2" t="n">
@@ -2985,7 +2981,7 @@
       <c r="B89" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="C89" s="3" t="s">
         <v>177</v>
       </c>
       <c r="D89" s="2" t="n">
@@ -2999,7 +2995,7 @@
       <c r="B90" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="C90" s="4" t="s">
+      <c r="C90" s="3" t="s">
         <v>179</v>
       </c>
       <c r="D90" s="2" t="n">
@@ -3013,7 +3009,7 @@
       <c r="B91" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="C91" s="4" t="s">
+      <c r="C91" s="3" t="s">
         <v>181</v>
       </c>
       <c r="D91" s="2" t="n">
@@ -3027,7 +3023,7 @@
       <c r="B92" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C92" s="4" t="s">
+      <c r="C92" s="3" t="s">
         <v>183</v>
       </c>
       <c r="D92" s="2" t="n">
@@ -3041,7 +3037,7 @@
       <c r="B93" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C93" s="4" t="s">
+      <c r="C93" s="3" t="s">
         <v>185</v>
       </c>
       <c r="D93" s="2" t="n">
@@ -3055,7 +3051,7 @@
       <c r="B94" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C94" s="4" t="s">
+      <c r="C94" s="3" t="s">
         <v>187</v>
       </c>
       <c r="D94" s="2" t="n">
@@ -3069,7 +3065,7 @@
       <c r="B95" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C95" s="4" t="s">
+      <c r="C95" s="3" t="s">
         <v>189</v>
       </c>
       <c r="D95" s="2" t="n">
@@ -3083,7 +3079,7 @@
       <c r="B96" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C96" s="4" t="s">
+      <c r="C96" s="3" t="s">
         <v>191</v>
       </c>
       <c r="D96" s="2" t="n">
@@ -3097,7 +3093,7 @@
       <c r="B97" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="3" t="s">
         <v>193</v>
       </c>
       <c r="D97" s="2" t="n">
@@ -3111,7 +3107,7 @@
       <c r="B98" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C98" s="3" t="s">
         <v>195</v>
       </c>
       <c r="D98" s="2" t="n">
@@ -3125,7 +3121,7 @@
       <c r="B99" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C99" s="3" t="s">
         <v>197</v>
       </c>
       <c r="D99" s="2" t="n">
@@ -3139,7 +3135,7 @@
       <c r="B100" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C100" s="4" t="s">
+      <c r="C100" s="3" t="s">
         <v>199</v>
       </c>
       <c r="D100" s="2" t="n">
@@ -3153,7 +3149,7 @@
       <c r="B101" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C101" s="4" t="s">
+      <c r="C101" s="3" t="s">
         <v>201</v>
       </c>
       <c r="D101" s="2" t="n">
@@ -3167,7 +3163,7 @@
       <c r="B102" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="C102" s="4" t="s">
+      <c r="C102" s="3" t="s">
         <v>203</v>
       </c>
       <c r="D102" s="2" t="n">
@@ -3181,7 +3177,7 @@
       <c r="B103" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C103" s="3" t="s">
         <v>205</v>
       </c>
       <c r="D103" s="2" t="n">
@@ -3195,7 +3191,7 @@
       <c r="B104" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="C104" s="4" t="s">
+      <c r="C104" s="3" t="s">
         <v>207</v>
       </c>
       <c r="D104" s="2" t="n">
@@ -3209,7 +3205,7 @@
       <c r="B105" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C105" s="4" t="s">
+      <c r="C105" s="3" t="s">
         <v>209</v>
       </c>
       <c r="D105" s="2" t="n">
@@ -3223,7 +3219,7 @@
       <c r="B106" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="C106" s="4" t="s">
+      <c r="C106" s="3" t="s">
         <v>211</v>
       </c>
       <c r="D106" s="2" t="n">
@@ -3237,7 +3233,7 @@
       <c r="B107" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="C107" s="4" t="s">
+      <c r="C107" s="3" t="s">
         <v>213</v>
       </c>
       <c r="D107" s="2" t="n">
@@ -3251,7 +3247,7 @@
       <c r="B108" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C108" s="4" t="s">
+      <c r="C108" s="3" t="s">
         <v>215</v>
       </c>
       <c r="D108" s="2" t="n">
@@ -3265,7 +3261,7 @@
       <c r="B109" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="C109" s="4" t="s">
+      <c r="C109" s="3" t="s">
         <v>217</v>
       </c>
       <c r="D109" s="2" t="n">
@@ -3279,7 +3275,7 @@
       <c r="B110" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="C110" s="4" t="s">
+      <c r="C110" s="3" t="s">
         <v>219</v>
       </c>
       <c r="D110" s="2" t="n">
@@ -3293,7 +3289,7 @@
       <c r="B111" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="C111" s="4" t="s">
+      <c r="C111" s="3" t="s">
         <v>221</v>
       </c>
       <c r="D111" s="2" t="n">
@@ -3307,7 +3303,7 @@
       <c r="B112" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="C112" s="4" t="s">
+      <c r="C112" s="3" t="s">
         <v>223</v>
       </c>
       <c r="D112" s="2" t="n">
@@ -3321,7 +3317,7 @@
       <c r="B113" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="C113" s="4" t="s">
+      <c r="C113" s="3" t="s">
         <v>225</v>
       </c>
       <c r="D113" s="2" t="n">
@@ -3335,7 +3331,7 @@
       <c r="B114" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="C114" s="4" t="s">
+      <c r="C114" s="3" t="s">
         <v>227</v>
       </c>
       <c r="D114" s="2" t="n">
@@ -3349,7 +3345,7 @@
       <c r="B115" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C115" s="4" t="s">
+      <c r="C115" s="3" t="s">
         <v>229</v>
       </c>
       <c r="D115" s="2" t="n">
@@ -3363,7 +3359,7 @@
       <c r="B116" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C116" s="3" t="s">
         <v>231</v>
       </c>
       <c r="D116" s="2" t="n">
@@ -3377,7 +3373,7 @@
       <c r="B117" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="C117" s="4" t="s">
+      <c r="C117" s="3" t="s">
         <v>233</v>
       </c>
       <c r="D117" s="2" t="n">
@@ -3391,7 +3387,7 @@
       <c r="B118" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="C118" s="4" t="s">
+      <c r="C118" s="3" t="s">
         <v>235</v>
       </c>
       <c r="D118" s="2" t="n">
@@ -3405,7 +3401,7 @@
       <c r="B119" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="C119" s="4" t="s">
+      <c r="C119" s="3" t="s">
         <v>237</v>
       </c>
       <c r="D119" s="2" t="n">
@@ -3419,7 +3415,7 @@
       <c r="B120" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="C120" s="4" t="s">
+      <c r="C120" s="3" t="s">
         <v>239</v>
       </c>
       <c r="D120" s="2" t="n">
@@ -3433,7 +3429,7 @@
       <c r="B121" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="C121" s="4" t="s">
+      <c r="C121" s="3" t="s">
         <v>241</v>
       </c>
       <c r="D121" s="2" t="n">
@@ -3447,7 +3443,7 @@
       <c r="B122" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="C122" s="4" t="s">
+      <c r="C122" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D122" s="2" t="n">
@@ -3461,7 +3457,7 @@
       <c r="B123" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="C123" s="4" t="s">
+      <c r="C123" s="3" t="s">
         <v>245</v>
       </c>
       <c r="D123" s="2" t="n">
@@ -3475,7 +3471,7 @@
       <c r="B124" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="C124" s="4" t="s">
+      <c r="C124" s="3" t="s">
         <v>247</v>
       </c>
       <c r="D124" s="2" t="n">
@@ -3489,7 +3485,7 @@
       <c r="B125" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C125" s="4" t="s">
+      <c r="C125" s="3" t="s">
         <v>249</v>
       </c>
       <c r="D125" s="2" t="n">
@@ -3503,7 +3499,7 @@
       <c r="B126" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="C126" s="4" t="s">
+      <c r="C126" s="3" t="s">
         <v>251</v>
       </c>
       <c r="D126" s="2" t="n">
@@ -3517,7 +3513,7 @@
       <c r="B127" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="C127" s="4" t="s">
+      <c r="C127" s="3" t="s">
         <v>253</v>
       </c>
       <c r="D127" s="2" t="n">
@@ -3531,7 +3527,7 @@
       <c r="B128" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="C128" s="4" t="s">
+      <c r="C128" s="3" t="s">
         <v>255</v>
       </c>
       <c r="D128" s="2" t="n">
@@ -3545,7 +3541,7 @@
       <c r="B129" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="C129" s="4" t="s">
+      <c r="C129" s="3" t="s">
         <v>257</v>
       </c>
       <c r="D129" s="2" t="n">
@@ -3559,7 +3555,7 @@
       <c r="B130" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C130" s="4" t="s">
+      <c r="C130" s="3" t="s">
         <v>259</v>
       </c>
       <c r="D130" s="2" t="n">
@@ -3573,7 +3569,7 @@
       <c r="B131" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C131" s="4" t="s">
+      <c r="C131" s="3" t="s">
         <v>261</v>
       </c>
       <c r="D131" s="2" t="n">
@@ -3587,7 +3583,7 @@
       <c r="B132" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="C132" s="4" t="s">
+      <c r="C132" s="3" t="s">
         <v>263</v>
       </c>
       <c r="D132" s="2" t="n">
@@ -3601,7 +3597,7 @@
       <c r="B133" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="C133" s="4" t="s">
+      <c r="C133" s="3" t="s">
         <v>265</v>
       </c>
       <c r="D133" s="2" t="n">
@@ -3615,7 +3611,7 @@
       <c r="B134" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="C134" s="4" t="s">
+      <c r="C134" s="3" t="s">
         <v>267</v>
       </c>
       <c r="D134" s="2" t="n">
@@ -3629,7 +3625,7 @@
       <c r="B135" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="C135" s="4" t="s">
+      <c r="C135" s="3" t="s">
         <v>269</v>
       </c>
       <c r="D135" s="2" t="n">
@@ -3643,7 +3639,7 @@
       <c r="B136" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="C136" s="4" t="s">
+      <c r="C136" s="3" t="s">
         <v>271</v>
       </c>
       <c r="D136" s="2" t="n">
@@ -3657,7 +3653,7 @@
       <c r="B137" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="C137" s="4" t="s">
+      <c r="C137" s="3" t="s">
         <v>273</v>
       </c>
       <c r="D137" s="2" t="n">
@@ -3671,7 +3667,7 @@
       <c r="B138" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="C138" s="4" t="s">
+      <c r="C138" s="3" t="s">
         <v>275</v>
       </c>
       <c r="D138" s="2" t="n">
@@ -3685,7 +3681,7 @@
       <c r="B139" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="C139" s="4" t="s">
+      <c r="C139" s="3" t="s">
         <v>277</v>
       </c>
       <c r="D139" s="2" t="n">
@@ -3699,7 +3695,7 @@
       <c r="B140" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="C140" s="4" t="s">
+      <c r="C140" s="3" t="s">
         <v>279</v>
       </c>
       <c r="D140" s="2" t="n">
@@ -3713,7 +3709,7 @@
       <c r="B141" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="C141" s="4" t="s">
+      <c r="C141" s="3" t="s">
         <v>281</v>
       </c>
       <c r="D141" s="2" t="n">
@@ -3727,7 +3723,7 @@
       <c r="B142" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="C142" s="4" t="s">
+      <c r="C142" s="3" t="s">
         <v>283</v>
       </c>
       <c r="D142" s="2" t="n">
@@ -3741,7 +3737,7 @@
       <c r="B143" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="C143" s="4" t="s">
+      <c r="C143" s="3" t="s">
         <v>285</v>
       </c>
       <c r="D143" s="2" t="n">
@@ -3755,7 +3751,7 @@
       <c r="B144" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="C144" s="4" t="s">
+      <c r="C144" s="3" t="s">
         <v>287</v>
       </c>
       <c r="D144" s="2" t="n">
@@ -3769,7 +3765,7 @@
       <c r="B145" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C145" s="4" t="s">
+      <c r="C145" s="3" t="s">
         <v>289</v>
       </c>
       <c r="D145" s="2" t="n">
@@ -3783,7 +3779,7 @@
       <c r="B146" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="C146" s="4" t="s">
+      <c r="C146" s="3" t="s">
         <v>291</v>
       </c>
       <c r="D146" s="2" t="n">
@@ -3797,7 +3793,7 @@
       <c r="B147" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="C147" s="4" t="s">
+      <c r="C147" s="3" t="s">
         <v>293</v>
       </c>
       <c r="D147" s="2" t="n">
@@ -3811,7 +3807,7 @@
       <c r="B148" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="C148" s="4" t="s">
+      <c r="C148" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D148" s="2" t="n">
@@ -3825,7 +3821,7 @@
       <c r="B149" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="C149" s="4" t="s">
+      <c r="C149" s="3" t="s">
         <v>297</v>
       </c>
       <c r="D149" s="2" t="n">
@@ -3839,7 +3835,7 @@
       <c r="B150" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="C150" s="4" t="s">
+      <c r="C150" s="3" t="s">
         <v>299</v>
       </c>
       <c r="D150" s="2" t="n">
@@ -3853,7 +3849,7 @@
       <c r="B151" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="C151" s="4" t="s">
+      <c r="C151" s="3" t="s">
         <v>301</v>
       </c>
       <c r="D151" s="2" t="n">
@@ -3867,7 +3863,7 @@
       <c r="B152" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="C152" s="4" t="s">
+      <c r="C152" s="3" t="s">
         <v>303</v>
       </c>
       <c r="D152" s="2" t="n">
@@ -3881,7 +3877,7 @@
       <c r="B153" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="C153" s="4" t="s">
+      <c r="C153" s="3" t="s">
         <v>305</v>
       </c>
       <c r="D153" s="2" t="n">
@@ -3895,7 +3891,7 @@
       <c r="B154" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="C154" s="4" t="s">
+      <c r="C154" s="3" t="s">
         <v>307</v>
       </c>
       <c r="D154" s="2" t="n">
@@ -3909,7 +3905,7 @@
       <c r="B155" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="C155" s="4" t="s">
+      <c r="C155" s="3" t="s">
         <v>309</v>
       </c>
       <c r="D155" s="2" t="n">
@@ -3923,7 +3919,7 @@
       <c r="B156" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="C156" s="4" t="s">
+      <c r="C156" s="3" t="s">
         <v>311</v>
       </c>
       <c r="D156" s="2" t="n">
@@ -3937,7 +3933,7 @@
       <c r="B157" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="C157" s="4" t="s">
+      <c r="C157" s="3" t="s">
         <v>313</v>
       </c>
       <c r="D157" s="2" t="n">
@@ -3951,7 +3947,7 @@
       <c r="B158" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="C158" s="4" t="s">
+      <c r="C158" s="3" t="s">
         <v>315</v>
       </c>
       <c r="D158" s="2" t="n">
@@ -3965,7 +3961,7 @@
       <c r="B159" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C159" s="4" t="s">
+      <c r="C159" s="3" t="s">
         <v>317</v>
       </c>
       <c r="D159" s="2" t="n">
@@ -3979,7 +3975,7 @@
       <c r="B160" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="C160" s="4" t="s">
+      <c r="C160" s="3" t="s">
         <v>319</v>
       </c>
       <c r="D160" s="2" t="n">
@@ -3993,7 +3989,7 @@
       <c r="B161" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="C161" s="4" t="s">
+      <c r="C161" s="3" t="s">
         <v>321</v>
       </c>
       <c r="D161" s="2" t="n">
@@ -4007,7 +4003,7 @@
       <c r="B162" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="C162" s="4" t="s">
+      <c r="C162" s="3" t="s">
         <v>323</v>
       </c>
       <c r="D162" s="2" t="n">
@@ -4021,7 +4017,7 @@
       <c r="B163" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="C163" s="4" t="s">
+      <c r="C163" s="3" t="s">
         <v>325</v>
       </c>
       <c r="D163" s="2" t="n">
@@ -4035,7 +4031,7 @@
       <c r="B164" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="C164" s="4" t="s">
+      <c r="C164" s="3" t="s">
         <v>327</v>
       </c>
       <c r="D164" s="2" t="n">
@@ -4049,7 +4045,7 @@
       <c r="B165" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C165" s="4" t="s">
+      <c r="C165" s="3" t="s">
         <v>329</v>
       </c>
       <c r="D165" s="2" t="n">
@@ -4063,7 +4059,7 @@
       <c r="B166" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="C166" s="4" t="s">
+      <c r="C166" s="3" t="s">
         <v>331</v>
       </c>
       <c r="D166" s="2" t="n">
@@ -4077,7 +4073,7 @@
       <c r="B167" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="C167" s="4" t="s">
+      <c r="C167" s="3" t="s">
         <v>333</v>
       </c>
       <c r="D167" s="2" t="n">
@@ -4091,7 +4087,7 @@
       <c r="B168" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="C168" s="4" t="s">
+      <c r="C168" s="3" t="s">
         <v>335</v>
       </c>
       <c r="D168" s="2" t="n">
@@ -4105,7 +4101,7 @@
       <c r="B169" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="C169" s="4" t="s">
+      <c r="C169" s="3" t="s">
         <v>337</v>
       </c>
       <c r="D169" s="2" t="n">
@@ -4119,7 +4115,7 @@
       <c r="B170" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="C170" s="4" t="s">
+      <c r="C170" s="3" t="s">
         <v>339</v>
       </c>
       <c r="D170" s="2" t="n">
@@ -4133,7 +4129,7 @@
       <c r="B171" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="C171" s="4" t="s">
+      <c r="C171" s="3" t="s">
         <v>341</v>
       </c>
       <c r="D171" s="2" t="n">
@@ -4147,7 +4143,7 @@
       <c r="B172" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="C172" s="4" t="s">
+      <c r="C172" s="3" t="s">
         <v>343</v>
       </c>
       <c r="D172" s="2" t="n">
@@ -4161,7 +4157,7 @@
       <c r="B173" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="C173" s="4" t="s">
+      <c r="C173" s="3" t="s">
         <v>345</v>
       </c>
       <c r="D173" s="2" t="n">
@@ -4175,7 +4171,7 @@
       <c r="B174" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="C174" s="4" t="s">
+      <c r="C174" s="3" t="s">
         <v>347</v>
       </c>
       <c r="D174" s="2" t="n">
@@ -4189,7 +4185,7 @@
       <c r="B175" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="C175" s="4" t="s">
+      <c r="C175" s="3" t="s">
         <v>349</v>
       </c>
       <c r="D175" s="2" t="n">
@@ -4203,7 +4199,7 @@
       <c r="B176" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C176" s="4" t="s">
+      <c r="C176" s="3" t="s">
         <v>351</v>
       </c>
       <c r="D176" s="2" t="n">
@@ -4217,7 +4213,7 @@
       <c r="B177" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="C177" s="4" t="s">
+      <c r="C177" s="3" t="s">
         <v>353</v>
       </c>
       <c r="D177" s="2" t="n">
@@ -4231,7 +4227,7 @@
       <c r="B178" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="C178" s="4" t="s">
+      <c r="C178" s="3" t="s">
         <v>355</v>
       </c>
       <c r="D178" s="2" t="n">
@@ -4245,7 +4241,7 @@
       <c r="B179" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="C179" s="4" t="s">
+      <c r="C179" s="3" t="s">
         <v>357</v>
       </c>
       <c r="D179" s="2" t="n">
@@ -4259,7 +4255,7 @@
       <c r="B180" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="C180" s="4" t="s">
+      <c r="C180" s="3" t="s">
         <v>359</v>
       </c>
       <c r="D180" s="2" t="n">
@@ -4273,7 +4269,7 @@
       <c r="B181" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="C181" s="4" t="s">
+      <c r="C181" s="3" t="s">
         <v>361</v>
       </c>
       <c r="D181" s="2" t="n">
@@ -4287,7 +4283,7 @@
       <c r="B182" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="C182" s="4" t="s">
+      <c r="C182" s="3" t="s">
         <v>363</v>
       </c>
       <c r="D182" s="2" t="n">
@@ -4301,7 +4297,7 @@
       <c r="B183" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="C183" s="4" t="s">
+      <c r="C183" s="3" t="s">
         <v>365</v>
       </c>
       <c r="D183" s="2" t="n">
@@ -4315,7 +4311,7 @@
       <c r="B184" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="C184" s="4" t="s">
+      <c r="C184" s="3" t="s">
         <v>367</v>
       </c>
       <c r="D184" s="2" t="n">
@@ -4329,7 +4325,7 @@
       <c r="B185" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="C185" s="4" t="s">
+      <c r="C185" s="3" t="s">
         <v>369</v>
       </c>
       <c r="D185" s="2" t="n">
@@ -4343,7 +4339,7 @@
       <c r="B186" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="C186" s="4" t="s">
+      <c r="C186" s="3" t="s">
         <v>371</v>
       </c>
       <c r="D186" s="2" t="n">
@@ -4357,7 +4353,7 @@
       <c r="B187" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="C187" s="4" t="s">
+      <c r="C187" s="3" t="s">
         <v>373</v>
       </c>
       <c r="D187" s="2" t="n">
@@ -4371,7 +4367,7 @@
       <c r="B188" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="C188" s="4" t="s">
+      <c r="C188" s="3" t="s">
         <v>375</v>
       </c>
       <c r="D188" s="2" t="n">
@@ -4385,7 +4381,7 @@
       <c r="B189" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="C189" s="4" t="s">
+      <c r="C189" s="3" t="s">
         <v>377</v>
       </c>
       <c r="D189" s="2" t="n">
@@ -4399,7 +4395,7 @@
       <c r="B190" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="C190" s="4" t="s">
+      <c r="C190" s="3" t="s">
         <v>379</v>
       </c>
       <c r="D190" s="2" t="n">
@@ -4413,7 +4409,7 @@
       <c r="B191" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="C191" s="4" t="s">
+      <c r="C191" s="3" t="s">
         <v>381</v>
       </c>
       <c r="D191" s="2" t="n">
@@ -4427,7 +4423,7 @@
       <c r="B192" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="C192" s="4" t="s">
+      <c r="C192" s="3" t="s">
         <v>383</v>
       </c>
       <c r="D192" s="2" t="n">
@@ -4441,7 +4437,7 @@
       <c r="B193" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="C193" s="4" t="s">
+      <c r="C193" s="3" t="s">
         <v>385</v>
       </c>
       <c r="D193" s="2" t="n">
@@ -4455,7 +4451,7 @@
       <c r="B194" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="C194" s="4" t="s">
+      <c r="C194" s="3" t="s">
         <v>387</v>
       </c>
       <c r="D194" s="2" t="n">
@@ -4469,7 +4465,7 @@
       <c r="B195" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="C195" s="4" t="s">
+      <c r="C195" s="3" t="s">
         <v>389</v>
       </c>
       <c r="D195" s="2" t="n">
@@ -4483,7 +4479,7 @@
       <c r="B196" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="C196" s="4" t="s">
+      <c r="C196" s="3" t="s">
         <v>391</v>
       </c>
       <c r="D196" s="2" t="n">
@@ -4497,7 +4493,7 @@
       <c r="B197" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="C197" s="4" t="s">
+      <c r="C197" s="3" t="s">
         <v>393</v>
       </c>
       <c r="D197" s="2" t="n">
@@ -4511,7 +4507,7 @@
       <c r="B198" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="C198" s="4" t="s">
+      <c r="C198" s="3" t="s">
         <v>395</v>
       </c>
       <c r="D198" s="2" t="n">
@@ -4525,7 +4521,7 @@
       <c r="B199" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C199" s="4" t="s">
+      <c r="C199" s="3" t="s">
         <v>397</v>
       </c>
       <c r="D199" s="2" t="n">
@@ -4539,7 +4535,7 @@
       <c r="B200" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="C200" s="4" t="s">
+      <c r="C200" s="3" t="s">
         <v>399</v>
       </c>
       <c r="D200" s="2" t="n">
@@ -4553,7 +4549,7 @@
       <c r="B201" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="C201" s="4" t="s">
+      <c r="C201" s="3" t="s">
         <v>401</v>
       </c>
       <c r="D201" s="2" t="n">
@@ -4567,7 +4563,7 @@
       <c r="B202" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="C202" s="4" t="s">
+      <c r="C202" s="3" t="s">
         <v>403</v>
       </c>
       <c r="D202" s="2" t="n">
@@ -4581,7 +4577,7 @@
       <c r="B203" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="C203" s="4" t="s">
+      <c r="C203" s="3" t="s">
         <v>405</v>
       </c>
       <c r="D203" s="2" t="n">
@@ -4595,7 +4591,7 @@
       <c r="B204" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="C204" s="4" t="s">
+      <c r="C204" s="3" t="s">
         <v>407</v>
       </c>
       <c r="D204" s="2" t="n">
@@ -4609,7 +4605,7 @@
       <c r="B205" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="C205" s="4" t="s">
+      <c r="C205" s="3" t="s">
         <v>409</v>
       </c>
       <c r="D205" s="2" t="n">
@@ -4623,7 +4619,7 @@
       <c r="B206" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="C206" s="4" t="s">
+      <c r="C206" s="3" t="s">
         <v>411</v>
       </c>
       <c r="D206" s="2" t="n">
@@ -4637,7 +4633,7 @@
       <c r="B207" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="C207" s="4" t="s">
+      <c r="C207" s="3" t="s">
         <v>413</v>
       </c>
       <c r="D207" s="2" t="n">
@@ -4651,7 +4647,7 @@
       <c r="B208" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="C208" s="4" t="s">
+      <c r="C208" s="3" t="s">
         <v>415</v>
       </c>
       <c r="D208" s="2" t="n">
@@ -4665,7 +4661,7 @@
       <c r="B209" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="C209" s="4" t="s">
+      <c r="C209" s="3" t="s">
         <v>417</v>
       </c>
       <c r="D209" s="2" t="n">
@@ -4679,7 +4675,7 @@
       <c r="B210" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="C210" s="4" t="s">
+      <c r="C210" s="3" t="s">
         <v>419</v>
       </c>
       <c r="D210" s="2" t="n">
@@ -4693,7 +4689,7 @@
       <c r="B211" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="C211" s="4" t="s">
+      <c r="C211" s="3" t="s">
         <v>421</v>
       </c>
       <c r="D211" s="2" t="n">
@@ -4707,7 +4703,7 @@
       <c r="B212" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="C212" s="4" t="s">
+      <c r="C212" s="3" t="s">
         <v>423</v>
       </c>
       <c r="D212" s="2" t="n">
@@ -4721,7 +4717,7 @@
       <c r="B213" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="C213" s="4" t="s">
+      <c r="C213" s="3" t="s">
         <v>425</v>
       </c>
       <c r="D213" s="2" t="n">
@@ -4735,7 +4731,7 @@
       <c r="B214" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="C214" s="4" t="s">
+      <c r="C214" s="3" t="s">
         <v>427</v>
       </c>
       <c r="D214" s="2" t="n">
@@ -4749,7 +4745,7 @@
       <c r="B215" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="C215" s="4" t="s">
+      <c r="C215" s="3" t="s">
         <v>429</v>
       </c>
       <c r="D215" s="2" t="n">
@@ -4763,7 +4759,7 @@
       <c r="B216" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="C216" s="4" t="s">
+      <c r="C216" s="3" t="s">
         <v>431</v>
       </c>
       <c r="D216" s="2" t="n">
@@ -4777,7 +4773,7 @@
       <c r="B217" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="C217" s="4" t="s">
+      <c r="C217" s="3" t="s">
         <v>433</v>
       </c>
       <c r="D217" s="2" t="n">
@@ -4791,7 +4787,7 @@
       <c r="B218" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C218" s="4" t="s">
+      <c r="C218" s="3" t="s">
         <v>435</v>
       </c>
       <c r="D218" s="2" t="n">
@@ -4805,7 +4801,7 @@
       <c r="B219" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="C219" s="4" t="s">
+      <c r="C219" s="3" t="s">
         <v>437</v>
       </c>
       <c r="D219" s="2" t="n">
@@ -4819,7 +4815,7 @@
       <c r="B220" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="C220" s="4" t="s">
+      <c r="C220" s="3" t="s">
         <v>439</v>
       </c>
       <c r="D220" s="2" t="n">
@@ -4833,7 +4829,7 @@
       <c r="B221" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="C221" s="4" t="s">
+      <c r="C221" s="3" t="s">
         <v>441</v>
       </c>
       <c r="D221" s="2" t="n">
@@ -4847,7 +4843,7 @@
       <c r="B222" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="C222" s="4" t="s">
+      <c r="C222" s="3" t="s">
         <v>443</v>
       </c>
       <c r="D222" s="2" t="n">
@@ -4861,7 +4857,7 @@
       <c r="B223" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="C223" s="4" t="s">
+      <c r="C223" s="3" t="s">
         <v>445</v>
       </c>
       <c r="D223" s="2" t="n">
@@ -4875,7 +4871,7 @@
       <c r="B224" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="C224" s="4" t="s">
+      <c r="C224" s="3" t="s">
         <v>447</v>
       </c>
       <c r="D224" s="2" t="n">
@@ -4889,7 +4885,7 @@
       <c r="B225" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="C225" s="4" t="s">
+      <c r="C225" s="3" t="s">
         <v>449</v>
       </c>
       <c r="D225" s="2" t="n">
@@ -4903,7 +4899,7 @@
       <c r="B226" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="C226" s="4" t="s">
+      <c r="C226" s="3" t="s">
         <v>451</v>
       </c>
       <c r="D226" s="2" t="n">
@@ -4917,7 +4913,7 @@
       <c r="B227" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="C227" s="4" t="s">
+      <c r="C227" s="3" t="s">
         <v>453</v>
       </c>
       <c r="D227" s="2" t="n">
@@ -4931,7 +4927,7 @@
       <c r="B228" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="C228" s="4" t="s">
+      <c r="C228" s="3" t="s">
         <v>455</v>
       </c>
       <c r="D228" s="2" t="n">
@@ -4945,7 +4941,7 @@
       <c r="B229" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="C229" s="4" t="s">
+      <c r="C229" s="3" t="s">
         <v>457</v>
       </c>
       <c r="D229" s="2" t="n">
@@ -4959,7 +4955,7 @@
       <c r="B230" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="C230" s="4" t="s">
+      <c r="C230" s="3" t="s">
         <v>459</v>
       </c>
       <c r="D230" s="2" t="n">
@@ -4973,7 +4969,7 @@
       <c r="B231" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="C231" s="4" t="s">
+      <c r="C231" s="3" t="s">
         <v>461</v>
       </c>
       <c r="D231" s="2" t="n">
@@ -4987,7 +4983,7 @@
       <c r="B232" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="C232" s="4" t="s">
+      <c r="C232" s="3" t="s">
         <v>463</v>
       </c>
       <c r="D232" s="2" t="n">
@@ -5001,7 +4997,7 @@
       <c r="B233" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="C233" s="4" t="s">
+      <c r="C233" s="3" t="s">
         <v>465</v>
       </c>
       <c r="D233" s="2" t="n">
@@ -5015,7 +5011,7 @@
       <c r="B234" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="C234" s="4" t="s">
+      <c r="C234" s="3" t="s">
         <v>467</v>
       </c>
       <c r="D234" s="2" t="n">
@@ -5029,7 +5025,7 @@
       <c r="B235" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="C235" s="4" t="s">
+      <c r="C235" s="3" t="s">
         <v>469</v>
       </c>
       <c r="D235" s="2" t="n">
@@ -5043,7 +5039,7 @@
       <c r="B236" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="C236" s="4" t="s">
+      <c r="C236" s="3" t="s">
         <v>471</v>
       </c>
       <c r="D236" s="2" t="n">
@@ -5057,7 +5053,7 @@
       <c r="B237" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="C237" s="4" t="s">
+      <c r="C237" s="3" t="s">
         <v>473</v>
       </c>
       <c r="D237" s="2" t="n">
@@ -5071,7 +5067,7 @@
       <c r="B238" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="C238" s="4" t="s">
+      <c r="C238" s="3" t="s">
         <v>475</v>
       </c>
       <c r="D238" s="2" t="n">
@@ -5085,7 +5081,7 @@
       <c r="B239" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="C239" s="4" t="s">
+      <c r="C239" s="3" t="s">
         <v>477</v>
       </c>
       <c r="D239" s="2" t="n">
@@ -5099,7 +5095,7 @@
       <c r="B240" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="C240" s="4" t="s">
+      <c r="C240" s="3" t="s">
         <v>479</v>
       </c>
       <c r="D240" s="2" t="n">
@@ -5113,7 +5109,7 @@
       <c r="B241" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="C241" s="4" t="s">
+      <c r="C241" s="3" t="s">
         <v>481</v>
       </c>
       <c r="D241" s="2" t="n">
@@ -5127,7 +5123,7 @@
       <c r="B242" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="C242" s="4" t="s">
+      <c r="C242" s="3" t="s">
         <v>483</v>
       </c>
       <c r="D242" s="2" t="n">
@@ -5141,7 +5137,7 @@
       <c r="B243" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="C243" s="4" t="s">
+      <c r="C243" s="3" t="s">
         <v>485</v>
       </c>
       <c r="D243" s="2" t="n">
@@ -5155,7 +5151,7 @@
       <c r="B244" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="C244" s="4" t="s">
+      <c r="C244" s="3" t="s">
         <v>487</v>
       </c>
       <c r="D244" s="2" t="n">
@@ -5169,7 +5165,7 @@
       <c r="B245" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="C245" s="4" t="s">
+      <c r="C245" s="3" t="s">
         <v>489</v>
       </c>
       <c r="D245" s="2" t="n">
@@ -5183,7 +5179,7 @@
       <c r="B246" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="C246" s="4" t="s">
+      <c r="C246" s="3" t="s">
         <v>491</v>
       </c>
       <c r="D246" s="2" t="n">
@@ -5197,7 +5193,7 @@
       <c r="B247" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="C247" s="4" t="s">
+      <c r="C247" s="3" t="s">
         <v>493</v>
       </c>
       <c r="D247" s="2" t="n">
@@ -5211,7 +5207,7 @@
       <c r="B248" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="C248" s="4" t="s">
+      <c r="C248" s="3" t="s">
         <v>495</v>
       </c>
       <c r="D248" s="2" t="n">
@@ -5225,7 +5221,7 @@
       <c r="B249" s="1" t="s">
         <v>496</v>
       </c>
-      <c r="C249" s="4" t="s">
+      <c r="C249" s="3" t="s">
         <v>497</v>
       </c>
       <c r="D249" s="2" t="n">
@@ -5239,7 +5235,7 @@
       <c r="B250" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="C250" s="4" t="s">
+      <c r="C250" s="3" t="s">
         <v>499</v>
       </c>
       <c r="D250" s="2" t="n">
@@ -5253,7 +5249,7 @@
       <c r="B251" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="C251" s="4" t="s">
+      <c r="C251" s="3" t="s">
         <v>501</v>
       </c>
       <c r="D251" s="2" t="n">
@@ -5261,7 +5257,6 @@
       </c>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C252" s="0"/>
       <c r="D252" s="2"/>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>